<commit_message>
Site updated: 2023-12-27 08:07:10
</commit_message>
<xml_diff>
--- a/1.xlsx
+++ b/1.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -831,6 +832,175 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>144780</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>587375</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="图片 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4411980" y="274320"/>
+          <a:ext cx="6538595" cy="3619500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>199390</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>37465</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="图片 12" descr="3233c127cbda2f7b96848122abb904b"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="199390" y="220980"/>
+          <a:ext cx="4105275" cy="3695700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>251460</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>117475</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="图片 4"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="251460" y="4488180"/>
+          <a:ext cx="3489960" cy="1938655"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>556895</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>39370</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="图片 5"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3672840" y="4465320"/>
+          <a:ext cx="4808855" cy="1883410"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1119,4 +1289,16 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="13.8"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>